<commit_message>
Working contact form, updated collages and Dynapac/Yanmar cards
- Form sends requests to a Google Apps Script web app: row in a Google Sheet
  plus an email notification (tools/form/Code.gs, step-by-step in FORM.md);
  honeypot field, error message with phone and email when sending fails
- Brand and industry collages rebuilt from the new Figma layouts; crop.mjs now
  locates frames on the board itself, so moving them in Figma no longer breaks it
- Portfolio cards: new photos for Dynapac and Yanmar
- Figma boards moved to media/layout

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bayern.xlsx
+++ b/bayern.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21190" windowHeight="13120"/>
+    <workbookView windowWidth="24750" windowHeight="12000"/>
   </bookViews>
   <sheets>
     <sheet name="bayern" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
   <si>
     <t>catalog path</t>
   </si>
@@ -41,6 +41,9 @@
     <t>card picture number</t>
   </si>
   <si>
+    <t>Contact information</t>
+  </si>
+  <si>
     <t>weber mt</t>
   </si>
   <si>
@@ -50,6 +53,12 @@
     <t>#0082c7</t>
   </si>
   <si>
+    <t xml:space="preserve">phone </t>
+  </si>
+  <si>
+    <t>+374 55 105500</t>
+  </si>
+  <si>
     <t xml:space="preserve">enar </t>
   </si>
   <si>
@@ -59,6 +68,12 @@
     <t>#fea904</t>
   </si>
   <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>info@bayern.am</t>
+  </si>
+  <si>
     <t>Geda</t>
   </si>
   <si>
@@ -68,6 +83,12 @@
     <t>#6078a3</t>
   </si>
   <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>Yerevan, Azatutyan ave. 24/15</t>
+  </si>
+  <si>
     <t>Hatz</t>
   </si>
   <si>
@@ -77,6 +98,9 @@
     <t>da281b</t>
   </si>
   <si>
+    <t>watsup</t>
+  </si>
+  <si>
     <t>Dynapac</t>
   </si>
   <si>
@@ -86,6 +110,12 @@
     <t>#941818</t>
   </si>
   <si>
+    <t>instagramm</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/bayernarmenia/</t>
+  </si>
+  <si>
     <t>Imer</t>
   </si>
   <si>
@@ -93,6 +123,12 @@
   </si>
   <si>
     <t>#579f97</t>
+  </si>
+  <si>
+    <t>facebook</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/profile.php?id=61562184064613&amp;ref=PROFILE_EDIT_xav_ig_profile_page_web#</t>
   </si>
   <si>
     <t>Ofmer</t>
@@ -810,7 +846,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -829,6 +865,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -848,6 +887,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1738,16 +1780,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="36.7272727272727" customWidth="1"/>
     <col min="8" max="8" width="16.8181818181818" customWidth="1"/>
     <col min="9" max="9" width="15.4545454545455" customWidth="1"/>
     <col min="11" max="11" width="12.4545454545455" customWidth="1"/>
+    <col min="14" max="14" width="15.7272727272727" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" spans="1:12">
+    <row r="1" ht="18" customHeight="1" spans="1:15">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1" t="s">
@@ -1768,14 +1811,17 @@
         <v>3</v>
       </c>
       <c r="L1" s="1"/>
+      <c r="N1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" ht="81" customHeight="1" spans="1:12">
+    <row r="2" ht="81" customHeight="1" spans="1:15">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1784,20 +1830,26 @@
       <c r="H2" s="1"/>
       <c r="I2" s="3"/>
       <c r="J2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K2" s="2">
         <v>3</v>
       </c>
       <c r="L2" s="1"/>
+      <c r="N2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="14" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" ht="81" customHeight="1" spans="1:12">
+    <row r="3" ht="81" customHeight="1" spans="1:15">
       <c r="A3" s="4"/>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1806,161 +1858,191 @@
       <c r="H3" s="1"/>
       <c r="I3" s="5"/>
       <c r="J3" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K3" s="2">
         <v>3</v>
       </c>
       <c r="L3" s="1"/>
+      <c r="N3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="4" ht="81" customHeight="1" spans="1:12">
+    <row r="4" ht="81" customHeight="1" spans="1:15">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="6"/>
+      <c r="I4" s="7"/>
       <c r="J4" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="K4" s="2">
         <v>3</v>
       </c>
       <c r="L4" s="1"/>
+      <c r="N4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="5" ht="81" customHeight="1" spans="1:12">
-      <c r="A5" s="7"/>
+    <row r="5" ht="81" customHeight="1" spans="1:15">
+      <c r="A5" s="8"/>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
-      <c r="I5" s="7"/>
+      <c r="I5" s="8"/>
       <c r="J5" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="K5" s="2">
         <v>2</v>
       </c>
       <c r="L5" s="1"/>
+      <c r="N5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O5" s="14" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="6" ht="81" customHeight="1" spans="1:12">
-      <c r="A6" s="8"/>
+    <row r="6" ht="81" customHeight="1" spans="1:15">
+      <c r="A6" s="9"/>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
-      <c r="I6" s="8"/>
+      <c r="I6" s="9"/>
       <c r="J6" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="K6" s="2">
         <v>3</v>
       </c>
       <c r="L6" s="1"/>
+      <c r="N6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="7" ht="81" customHeight="1" spans="1:12">
+    <row r="7" ht="81" customHeight="1" spans="1:15">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-      <c r="I7" s="9"/>
+      <c r="I7" s="10"/>
       <c r="J7" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="K7" s="2">
         <v>3</v>
       </c>
       <c r="L7" s="1"/>
+      <c r="N7" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="8" ht="81" customHeight="1" spans="1:12">
-      <c r="A8" s="10"/>
+    <row r="8" ht="81" customHeight="1" spans="1:15">
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="10"/>
+      <c r="I8" s="11"/>
       <c r="J8" s="2" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="K8" s="2">
         <v>3</v>
       </c>
       <c r="L8" s="1"/>
     </row>
-    <row r="9" ht="93" customHeight="1" spans="1:12">
+    <row r="9" ht="93" customHeight="1" spans="1:15">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
-      <c r="I9" s="11"/>
+      <c r="I9" s="12"/>
       <c r="J9" s="2" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="K9" s="2">
         <v>3</v>
       </c>
       <c r="L9" s="1"/>
     </row>
-    <row r="10" ht="81" customHeight="1" spans="1:12">
+    <row r="10" ht="81" customHeight="1" spans="1:15">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
-      <c r="I10" s="12"/>
+      <c r="I10" s="13"/>
       <c r="J10" s="2" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K10" s="2">
         <v>3</v>
@@ -1970,6 +2052,11 @@
     <row r="11" ht="18" customHeight="1"/>
     <row r="12" ht="18" customHeight="1"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="O3" r:id="rId2" display="info@bayern.am"/>
+    <hyperlink ref="O7" r:id="rId3" display="https://www.facebook.com/profile.php?id=61562184064613&amp;ref=PROFILE_EDIT_xav_ig_profile_page_web#"/>
+    <hyperlink ref="O6" r:id="rId4" display="https://www.instagram.com/bayernarmenia/"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>

</xml_diff>